<commit_message>
feat: ajout images recettes, mise à jour fonctions et dépendances
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app_list/assets/recettes.xlsx
+++ b/app_list/assets/recettes.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\App\app_list\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47CB8665-D91D-4D79-92C2-B52C0B7C07F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A649EC49-2898-4A05-BCA8-3B90053B4301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D94F266F-8CD8-4294-A504-AA449366F284}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D94F266F-8CD8-4294-A504-AA449366F284}"/>
   </bookViews>
   <sheets>
     <sheet name="plats" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">plats!$A$1:$F$56</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">plats!$A$1:$F$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="128">
   <si>
     <t>Plat</t>
   </si>
@@ -308,6 +308,132 @@
   </si>
   <si>
     <t>assets/Images/pates_saucisseitalienne.jpg</t>
+  </si>
+  <si>
+    <t>assets/Images/chicken_finger.jpg</t>
+  </si>
+  <si>
+    <t>Chicken Fingers</t>
+  </si>
+  <si>
+    <t>Epices à poulet</t>
+  </si>
+  <si>
+    <t>Fécule de maïs</t>
+  </si>
+  <si>
+    <t>assets/Images/Moussaka.jpg</t>
+  </si>
+  <si>
+    <t>Moussaka</t>
+  </si>
+  <si>
+    <t>Lait</t>
+  </si>
+  <si>
+    <t>Beurre</t>
+  </si>
+  <si>
+    <t>Vin rouge</t>
+  </si>
+  <si>
+    <t>Boisson</t>
+  </si>
+  <si>
+    <t>assets/Images/risotto_chorizo.jpg</t>
+  </si>
+  <si>
+    <t>Risotto Chorizo</t>
+  </si>
+  <si>
+    <t>Risotto</t>
+  </si>
+  <si>
+    <t>Chorizo</t>
+  </si>
+  <si>
+    <t>Apéro</t>
+  </si>
+  <si>
+    <t>Vin Blanc</t>
+  </si>
+  <si>
+    <t>Cube de bouillons de poule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pcs </t>
+  </si>
+  <si>
+    <t>assets/Images/samossa.jpg</t>
+  </si>
+  <si>
+    <t>Samossa</t>
+  </si>
+  <si>
+    <t>Petit pois</t>
+  </si>
+  <si>
+    <t>Boite</t>
+  </si>
+  <si>
+    <t>Feuilles de brick</t>
+  </si>
+  <si>
+    <t>Frais</t>
+  </si>
+  <si>
+    <t>Curry</t>
+  </si>
+  <si>
+    <t>assets/Images/curry_vert.jpg</t>
+  </si>
+  <si>
+    <t>Curry Vert</t>
+  </si>
+  <si>
+    <t>Brocoli</t>
+  </si>
+  <si>
+    <t>Bambou</t>
+  </si>
+  <si>
+    <t>Monde</t>
+  </si>
+  <si>
+    <t>assets/Images/pates_ail.jpg</t>
+  </si>
+  <si>
+    <t>Pâtes à l'ail</t>
+  </si>
+  <si>
+    <t>assets/Images/pain_saucisse.jpg</t>
+  </si>
+  <si>
+    <t>Baguette</t>
+  </si>
+  <si>
+    <t>Pain saucisse</t>
+  </si>
+  <si>
+    <t>Saucisses de campagne</t>
+  </si>
+  <si>
+    <t>Salade</t>
+  </si>
+  <si>
+    <t>assets/Images/pates_vodka.jpg</t>
+  </si>
+  <si>
+    <t>Pâtes Vodka</t>
+  </si>
+  <si>
+    <t>Vodka</t>
+  </si>
+  <si>
+    <t>cl</t>
+  </si>
+  <si>
+    <t>Dés de lardon fumé</t>
   </si>
 </sst>
 </file>
@@ -323,7 +449,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -333,6 +459,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -349,11 +481,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,8 +536,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A4F2E1D6-736A-49AE-9DF0-D90176966E20}" name="plats" displayName="plats" ref="A1:F56" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:F56" xr:uid="{A4F2E1D6-736A-49AE-9DF0-D90176966E20}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A4F2E1D6-736A-49AE-9DF0-D90176966E20}" name="plats" displayName="plats" ref="A1:F96" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:F96" xr:uid="{A4F2E1D6-736A-49AE-9DF0-D90176966E20}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{68CB759F-945C-4F2E-894C-159C544C9DCE}" uniqueName="1" name="Plat" queryTableFieldId="1" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{D23BF9A4-4548-405E-A536-AE3E04137B5D}" uniqueName="2" name="Ingrédient" queryTableFieldId="2" dataDxfId="3"/>
@@ -734,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{546FEE4A-874C-4410-8E97-8DF4AB8926DA}">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.08984375" customWidth="1"/>
@@ -766,483 +899,483 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="1">
         <v>150</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3">
         <v>150</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>28</v>
       </c>
       <c r="C4">
         <v>500</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
         <v>400</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
       <c r="C6">
         <v>8</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="1">
         <v>400</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>33</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>35</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>36</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>38</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="3">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>25</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>39</v>
       </c>
       <c r="C15">
         <v>3</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>26</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>27</v>
       </c>
       <c r="C17">
         <v>300</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>35</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="1" t="s">
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="1">
         <v>500</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>42</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="1" t="s">
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>44</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
         <v>45</v>
       </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B24" t="s">
         <v>46</v>
       </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" s="1" t="s">
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B25" t="s">
         <v>47</v>
       </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
         <v>48</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F25" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="3">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
@@ -1250,99 +1383,99 @@
         <v>49</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26">
-        <v>200</v>
+        <v>50</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27">
+        <v>200</v>
+      </c>
+      <c r="D27" t="s">
+        <v>4</v>
+      </c>
+      <c r="E27" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" t="s">
         <v>54</v>
       </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="1" t="s">
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B29" t="s">
         <v>55</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>500</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D29" t="s">
         <v>5</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E29" t="s">
         <v>56</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F29" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B30" t="s">
         <v>47</v>
       </c>
-      <c r="C29">
+      <c r="C30">
         <v>5</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="1" t="s">
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
         <v>48</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F30" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C30" s="3">
-        <v>250</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
@@ -1350,119 +1483,119 @@
         <v>64</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C31">
+        <v>57</v>
+      </c>
+      <c r="C31" s="1">
+        <v>250</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="E31" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
         <v>59</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>2</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="1" t="s">
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B34" t="s">
         <v>60</v>
       </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" s="1" t="s">
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" t="s">
         <v>29</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F34" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B35" t="s">
         <v>61</v>
       </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E34" s="1" t="s">
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" t="s">
         <v>29</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F35" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B36" t="s">
         <v>62</v>
       </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E35" s="1" t="s">
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" t="s">
         <v>29</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F36" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C36" s="3">
-        <v>330</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
@@ -1470,79 +1603,79 @@
         <v>65</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
+        <v>66</v>
+      </c>
+      <c r="C37" s="1">
+        <v>330</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
+      <c r="A38" t="s">
         <v>65</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" t="s">
         <v>68</v>
       </c>
-      <c r="C38">
+      <c r="C39">
         <v>50</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" t="s">
         <v>4</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E39" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F39" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>65</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" t="s">
         <v>69</v>
       </c>
-      <c r="C39">
+      <c r="C40">
         <v>100</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D40" t="s">
         <v>4</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E40" t="s">
         <v>15</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F40" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C40" s="3">
-        <v>250</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -1550,219 +1683,219 @@
         <v>71</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C41">
-        <v>2</v>
+        <v>72</v>
+      </c>
+      <c r="C41" s="1">
+        <v>250</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+      <c r="A42" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>71</v>
+      </c>
+      <c r="B43" t="s">
         <v>74</v>
-      </c>
-      <c r="C42">
-        <v>3</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F43" s="1" t="s">
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="1" t="s">
+      <c r="A44" t="s">
         <v>71</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44" t="s">
+        <v>7</v>
+      </c>
+      <c r="E44" t="s">
+        <v>23</v>
+      </c>
+      <c r="F44" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45" t="s">
         <v>26</v>
       </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F44" s="1" t="s">
+      <c r="C45">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E45" t="s">
+        <v>23</v>
+      </c>
+      <c r="F45" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B46" t="s">
         <v>33</v>
       </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F45" s="1" t="s">
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46" t="s">
+        <v>7</v>
+      </c>
+      <c r="E46" t="s">
+        <v>23</v>
+      </c>
+      <c r="F46" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>71</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B47" t="s">
         <v>76</v>
       </c>
-      <c r="C46">
+      <c r="C47">
         <v>100</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D47" t="s">
         <v>4</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E47" t="s">
         <v>29</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F47" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>71</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B48" t="s">
         <v>77</v>
       </c>
-      <c r="C47">
+      <c r="C48">
         <v>3</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E47" s="1" t="s">
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+      <c r="E48" t="s">
         <v>29</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F48" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" s="1" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B49" t="s">
         <v>78</v>
       </c>
-      <c r="C48">
+      <c r="C49">
         <v>100</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D49" t="s">
         <v>4</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E49" t="s">
         <v>29</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F49" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B50" t="s">
         <v>47</v>
       </c>
-      <c r="C49">
+      <c r="C50">
         <v>2</v>
       </c>
-      <c r="D49" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="1" t="s">
+      <c r="D50" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" t="s">
         <v>29</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F50" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>71</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B51" t="s">
         <v>79</v>
       </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" s="1" t="s">
+      <c r="C51">
+        <v>1</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" t="s">
         <v>29</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F51" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" s="3">
-        <v>330</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
@@ -1770,55 +1903,55 @@
         <v>81</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C52" s="1">
+        <v>330</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>81</v>
+      </c>
+      <c r="B53" t="s">
         <v>82</v>
-      </c>
-      <c r="C52">
-        <v>2</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A53" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C53">
         <v>2</v>
       </c>
-      <c r="D53" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>23</v>
+      <c r="D53" t="s">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>20</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
+      <c r="A54" t="s">
         <v>81</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>83</v>
+      <c r="B54" t="s">
+        <v>35</v>
       </c>
       <c r="C54">
-        <v>1</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E54" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D54" t="s">
+        <v>7</v>
+      </c>
+      <c r="E54" t="s">
         <v>23</v>
       </c>
       <c r="F54" s="2" t="s">
@@ -1826,43 +1959,843 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
+      <c r="A55" t="s">
         <v>81</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>55</v>
+      <c r="B55" t="s">
+        <v>83</v>
       </c>
       <c r="C55">
-        <v>100</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>7</v>
+      </c>
+      <c r="E55" t="s">
+        <v>23</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
+      <c r="A56" t="s">
         <v>81</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>84</v>
+      <c r="B56" t="s">
+        <v>55</v>
       </c>
       <c r="C56">
-        <v>1</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>29</v>
+        <v>100</v>
+      </c>
+      <c r="D56" t="s">
+        <v>5</v>
+      </c>
+      <c r="E56" t="s">
+        <v>56</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>81</v>
+      </c>
+      <c r="B57" t="s">
+        <v>84</v>
+      </c>
+      <c r="C57">
+        <v>1</v>
+      </c>
+      <c r="D57" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" t="s">
+        <v>29</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A58" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C58" s="1">
+        <v>2</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A60" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C60">
+        <v>2</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" s="1">
+        <v>500</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C63">
+        <v>2</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64">
+        <v>4</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C67">
+        <v>1</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C68">
+        <v>1</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C69">
+        <v>1</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C70" s="1">
+        <v>300</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C71">
+        <v>1</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C73">
+        <v>1</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C74">
+        <v>1</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" s="1">
+        <v>300</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C76">
+        <v>2</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C77">
+        <v>1</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C78">
+        <v>1</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C79">
+        <v>1</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C81" s="1">
+        <v>2</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C82">
+        <v>1</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C83">
+        <v>2</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A84" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C84">
+        <v>1</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C85">
+        <v>300</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C87" s="1">
+        <v>330</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C88">
+        <v>1</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C89">
+        <v>1</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C90" s="1">
+        <v>2</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C91">
+        <v>4</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C92">
+        <v>1</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C93" s="1">
+        <v>330</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C94">
+        <v>5</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C95">
+        <v>100</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C96">
+        <v>200</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>